<commit_message>
Fase 4: pontos de Organizacao
O placar e do servidor inteiro, nao de cada jogador: cada incursao credita a
Organizacao a que pertence. Uma run pontua em tres momentos -- cada sala
secundaria superada vale o que estiver na coluna nova da planilha, concluir o
objetivo vale o maior bonus (pontos_conclusao, por incursao) e levar a run ate
o fim rende a participacao configurada no .env, inclusive em derrota.

Cada motivo entra no placar uma vez so: o lancamento fica gravado com a run,
entao reprocessar uma sala nao infla o total. Ao fim da run o bot posta o
balanco, e /organizacao placar, extrato e ajustar cobrem consulta e correcao
manual do que aconteceu na mesa.

MEs continuam fora do bot, na planilha do Google Sheets: o embed final so
mostra quanto cada participante ganhou, sem guardar saldo por jogador.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/planilhas/incursao_exemplo.xlsx
+++ b/data/planilhas/incursao_exemplo.xlsx
@@ -287,6 +287,11 @@
     <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <t>Bônus da sala (texto livre). Opcional.</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <t>Pontos de Organizacao se a sala for superada. 0 ou vazio = nenhum.</t>
       </text>
     </comment>
   </commentList>
@@ -582,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -764,6 +769,30 @@
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Perícias válidas: veja a aba 'Pericias'. Pode escrever com ou sem acento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>Pontos de Organização</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Sao do servidor inteiro, nao de cada jogador. Completar o objetivo da 'pontos_conclusao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>(aba Incursao) e cada sala superada da o que estiver em 'pontos_organizacao'.</t>
         </is>
       </c>
     </row>
@@ -778,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -900,6 +929,21 @@
       <c r="C7" s="5" t="inlineStr">
         <is>
           <t>MEs por participante ao completar o objetivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>pontos_conclusao</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Pontos que o servidor ganha com a Organizacao ao completar o objetivo.</t>
         </is>
       </c>
     </row>
@@ -914,7 +958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -933,6 +977,7 @@
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="11" customWidth="1" min="15" max="15"/>
     <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1014,6 +1059,11 @@
       <c r="P1" s="3" t="inlineStr">
         <is>
           <t>recompensa</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>pontos_organizacao</t>
         </is>
       </c>
     </row>
@@ -1074,6 +1124,9 @@
           <t>Quem passa ileso encontra um fragmento do selo.</t>
         </is>
       </c>
+      <c r="Q2" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" ht="62" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -1132,6 +1185,9 @@
           <t>Revela a CA do chefe antes do confronto final.</t>
         </is>
       </c>
+      <c r="Q3" s="6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4" ht="62" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -1192,6 +1248,9 @@
         <v>26</v>
       </c>
       <c r="P4" s="6" t="inlineStr"/>
+      <c r="Q4" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" ht="62" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -1246,6 +1305,9 @@
       <c r="N5" s="6" t="inlineStr"/>
       <c r="O5" s="6" t="inlineStr"/>
       <c r="P5" s="6" t="inlineStr"/>
+      <c r="Q5" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" ht="62" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -1296,6 +1358,9 @@
           <t>Cada personagem caído volta com metade do HP máximo.</t>
         </is>
       </c>
+      <c r="Q6" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" ht="62" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -1354,6 +1419,9 @@
           <t>Materiais raros para quem passar no teste.</t>
         </is>
       </c>
+      <c r="Q7" s="6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8" ht="62" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -1414,6 +1482,9 @@
         <v>34</v>
       </c>
       <c r="P8" s="6" t="inlineStr"/>
+      <c r="Q8" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" ht="62" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -1472,6 +1543,9 @@
           <t>O chefe começa o combate final com 10 de HP a menos.</t>
         </is>
       </c>
+      <c r="Q9" s="6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10" ht="62" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -1526,6 +1600,9 @@
       <c r="N10" s="6" t="inlineStr"/>
       <c r="O10" s="6" t="inlineStr"/>
       <c r="P10" s="6" t="inlineStr"/>
+      <c r="Q10" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" ht="62" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
@@ -1591,6 +1668,9 @@
         <is>
           <t>10 MEs por participante + pontos com o Vórtice Oculto</t>
         </is>
+      </c>
+      <c r="Q11" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>